<commit_message>
y is auc for block wise
</commit_message>
<xml_diff>
--- a/eval_output/BASE_CIFAR_noniid0.1.xlsx
+++ b/eval_output/BASE_CIFAR_noniid0.1.xlsx
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>94882534094.33824</v>
+        <v>94919074238.21313</v>
       </c>
       <c r="D2" t="n">
         <v>528418784</v>
@@ -503,7 +503,7 @@
         <v>2119984768</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>57.60342336740561</v>
+        <v>57.62560697999166</v>
       </c>
       <c r="G2" t="n">
         <v>476754112</v>
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>94637080003.24731</v>
+        <v>94714971614.42912</v>
       </c>
       <c r="D3" t="n">
         <v>528512896</v>
@@ -536,7 +536,7 @@
         <v>2122557312</v>
       </c>
       <c r="F3" t="n">
-        <v>57.45440757581309</v>
+        <v>57.50169576745449</v>
       </c>
       <c r="G3" t="n">
         <v>476754112</v>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>95184023277.02496</v>
+        <v>95197419237.2735</v>
       </c>
       <c r="D4" t="n">
         <v>502500096</v>
@@ -569,7 +569,7 @@
         <v>2120142208</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>57.78645820302382</v>
+        <v>57.79459092394</v>
       </c>
       <c r="G4" t="n">
         <v>476754112</v>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>93302158560.4063</v>
+        <v>93405531147.70314</v>
       </c>
       <c r="D6" t="n">
         <v>477005408</v>
@@ -635,7 +635,7 @@
         <v>2121297408</v>
       </c>
       <c r="F6" t="n">
-        <v>56.64397343460703</v>
+        <v>56.70673119047308</v>
       </c>
       <c r="G6" t="n">
         <v>476754112</v>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>96921215337.34682</v>
+        <v>96968246457.59492</v>
       </c>
       <c r="D8" t="n">
         <v>528795200</v>
@@ -701,7 +701,7 @@
         <v>2119827200</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>58.84111184055969</v>
+        <v>58.86966455109756</v>
       </c>
       <c r="G8" t="n">
         <v>476754112</v>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>96322230557.80225</v>
+        <v>96472855499.27354</v>
       </c>
       <c r="D9" t="n">
         <v>528512896</v>
@@ -734,7 +734,7 @@
         <v>2122347392</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>58.47746668525184</v>
+        <v>58.56891146332486</v>
       </c>
       <c r="G9" t="n">
         <v>476754112</v>
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>95628649300.81828</v>
+        <v>95686666419.13348</v>
       </c>
       <c r="D10" t="n">
         <v>502633472</v>
@@ -767,7 +767,7 @@
         <v>2119039616</v>
       </c>
       <c r="F10" t="n">
-        <v>58.05639177228608</v>
+        <v>58.09161410968218</v>
       </c>
       <c r="G10" t="n">
         <v>476754112</v>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>95492827588.9628</v>
+        <v>95492890000.2765</v>
       </c>
       <c r="D11" t="n">
         <v>477172960</v>
@@ -800,7 +800,7 @@
         <v>2122294912</v>
       </c>
       <c r="F11" t="n">
-        <v>57.97393407187603</v>
+        <v>57.97397196194042</v>
       </c>
       <c r="G11" t="n">
         <v>476754112</v>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>95638291817.28784</v>
+        <v>95769850282.88489</v>
       </c>
       <c r="D12" t="n">
         <v>476754112</v>
@@ -833,7 +833,7 @@
         <v>2122189824</v>
       </c>
       <c r="F12" t="n">
-        <v>58.06224576811181</v>
+        <v>58.14211524107317</v>
       </c>
       <c r="G12" t="n">
         <v>476754112</v>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>63018847410.52349</v>
+        <v>63063356878.3103</v>
       </c>
       <c r="D2" t="n">
         <v>528418784</v>
@@ -960,7 +960,7 @@
         <v>1596734336</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.20248262564477</v>
+        <v>56.24217777547303</v>
       </c>
       <c r="G2" t="n">
         <v>476712224</v>
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>62766929990.88922</v>
+        <v>62805307350.7708</v>
       </c>
       <c r="D3" t="n">
         <v>528465824</v>
@@ -993,7 +993,7 @@
         <v>1596944256</v>
       </c>
       <c r="F3" t="n">
-        <v>55.97781357849669</v>
+        <v>56.01203989317223</v>
       </c>
       <c r="G3" t="n">
         <v>476712224</v>
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>62806333245.38968</v>
+        <v>62908339467.87598</v>
       </c>
       <c r="D4" t="n">
         <v>502500096</v>
@@ -1026,7 +1026,7 @@
         <v>1593584000</v>
       </c>
       <c r="F4" t="n">
-        <v>56.01295482302041</v>
+        <v>56.10392765388873</v>
       </c>
       <c r="G4" t="n">
         <v>476712224</v>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>62813758562.98936</v>
+        <v>62992095801.28742</v>
       </c>
       <c r="D5" t="n">
         <v>476712224</v>
@@ -1059,7 +1059,7 @@
         <v>1592954112</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>56.01957698925374</v>
+        <v>56.17862457499678</v>
       </c>
       <c r="G5" t="n">
         <v>476712224</v>
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>62058294036.44006</v>
+        <v>62092698855.19656</v>
       </c>
       <c r="D6" t="n">
         <v>476879744</v>
@@ -1092,7 +1092,7 @@
         <v>1596944256</v>
       </c>
       <c r="F6" t="n">
-        <v>55.34582645790734</v>
+        <v>55.37650991702878</v>
       </c>
       <c r="G6" t="n">
         <v>476712224</v>
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>64459355652.61506</v>
+        <v>64599920667.33306</v>
       </c>
       <c r="D8" t="n">
         <v>528654048</v>
@@ -1158,7 +1158,7 @@
         <v>1596734208</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>57.48717986742152</v>
+        <v>57.61254082088356</v>
       </c>
       <c r="G8" t="n">
         <v>476712224</v>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>63892469953.25922</v>
+        <v>63994081987.75257</v>
       </c>
       <c r="D9" t="n">
         <v>528465824</v>
@@ -1191,7 +1191,7 @@
         <v>1595684224</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>56.98161074043915</v>
+        <v>57.07223202022815</v>
       </c>
       <c r="G9" t="n">
         <v>476712224</v>
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>63354614803.34739</v>
+        <v>63491650716.78462</v>
       </c>
       <c r="D10" t="n">
         <v>502589024</v>
@@ -1224,7 +1224,7 @@
         <v>1594214144</v>
       </c>
       <c r="F10" t="n">
-        <v>56.50193210523477</v>
+        <v>56.62414567880069</v>
       </c>
       <c r="G10" t="n">
         <v>476712224</v>
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>63853134048.1697</v>
+        <v>63967102978.81035</v>
       </c>
       <c r="D11" t="n">
         <v>477131072</v>
@@ -1257,7 +1257,7 @@
         <v>1597994368</v>
       </c>
       <c r="F11" t="n">
-        <v>56.94652956055092</v>
+        <v>57.0481711663148</v>
       </c>
       <c r="G11" t="n">
         <v>476712224</v>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>63553387787.82253</v>
+        <v>63641389923.36529</v>
       </c>
       <c r="D12" t="n">
         <v>476712224</v>
@@ -1290,7 +1290,7 @@
         <v>1597994496</v>
       </c>
       <c r="F12" t="n">
-        <v>56.67920502699479</v>
+        <v>56.75768850768497</v>
       </c>
       <c r="G12" t="n">
         <v>476712224</v>
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>28573608495.61668</v>
+        <v>28701126251.50632</v>
       </c>
       <c r="D2" t="n">
         <v>528418784</v>
@@ -1417,7 +1417,7 @@
         <v>1072013888</v>
       </c>
       <c r="F2" t="n">
-        <v>47.755101264692</v>
+        <v>47.96822182125349</v>
       </c>
       <c r="G2" t="n">
         <v>476670336</v>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28554447907.21085</v>
+        <v>28630390483.81919</v>
       </c>
       <c r="D3" t="n">
         <v>528418784</v>
@@ -1450,7 +1450,7 @@
         <v>1074219008</v>
       </c>
       <c r="F3" t="n">
-        <v>47.72307815358401</v>
+        <v>47.85000105997118</v>
       </c>
       <c r="G3" t="n">
         <v>476670336</v>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28729568949.08359</v>
+        <v>29006937463.50329</v>
       </c>
       <c r="D4" t="n">
         <v>502500096</v>
@@ -1482,8 +1482,8 @@
       <c r="E4" t="n">
         <v>1072276288</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>48.01575813096573</v>
+      <c r="F4" s="2" t="n">
+        <v>48.47932441436959</v>
       </c>
       <c r="G4" t="n">
         <v>476670336</v>
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28616218784.97509</v>
+        <v>29036420285.93116</v>
       </c>
       <c r="D5" t="n">
         <v>476670336</v>
@@ -1515,8 +1515,8 @@
       <c r="E5" t="n">
         <v>1074534016</v>
       </c>
-      <c r="F5" s="2" t="n">
-        <v>47.82631588511843</v>
+      <c r="F5" s="3" t="n">
+        <v>48.52859908581431</v>
       </c>
       <c r="G5" t="n">
         <v>476670336</v>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27925186587.12053</v>
+        <v>28105041582.39169</v>
       </c>
       <c r="D6" t="n">
         <v>476754112</v>
@@ -1549,7 +1549,7 @@
         <v>1072276288</v>
       </c>
       <c r="F6" t="n">
-        <v>46.67139306216558</v>
+        <v>46.97198490073063</v>
       </c>
       <c r="G6" t="n">
         <v>476670336</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29358480520.07931</v>
+        <v>29424961615.27751</v>
       </c>
       <c r="D8" t="n">
         <v>528512864</v>
@@ -1614,8 +1614,8 @@
       <c r="E8" t="n">
         <v>1073221376</v>
       </c>
-      <c r="F8" s="3" t="n">
-        <v>49.06685868636266</v>
+      <c r="F8" s="2" t="n">
+        <v>49.17796860913858</v>
       </c>
       <c r="G8" t="n">
         <v>476670336</v>
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>29172574690.22541</v>
+        <v>29244986622.3396</v>
       </c>
       <c r="D9" t="n">
         <v>528418784</v>
@@ -1648,7 +1648,7 @@
         <v>1074166400</v>
       </c>
       <c r="F9" t="n">
-        <v>48.75615408173662</v>
+        <v>48.8771762183497</v>
       </c>
       <c r="G9" t="n">
         <v>476670336</v>
@@ -1672,7 +1672,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>29261259811.12676</v>
+        <v>29500887215.64862</v>
       </c>
       <c r="D10" t="n">
         <v>502544544</v>
@@ -1680,8 +1680,8 @@
       <c r="E10" t="n">
         <v>1074901504</v>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>48.90437361550553</v>
+      <c r="F10" s="3" t="n">
+        <v>49.30486314312303</v>
       </c>
       <c r="G10" t="n">
         <v>476670336</v>
@@ -1705,7 +1705,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>29009965953.67334</v>
+        <v>29271752656.7956</v>
       </c>
       <c r="D11" t="n">
         <v>476921664</v>
@@ -1714,7 +1714,7 @@
         <v>1074638976</v>
       </c>
       <c r="F11" t="n">
-        <v>48.48438593310537</v>
+        <v>48.92191031926303</v>
       </c>
       <c r="G11" t="n">
         <v>476670336</v>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>28950233352.14146</v>
+        <v>29143293157.91536</v>
       </c>
       <c r="D12" t="n">
         <v>476670336</v>
@@ -1747,7 +1747,7 @@
         <v>1072906368</v>
       </c>
       <c r="F12" t="n">
-        <v>48.38455477473433</v>
+        <v>48.70721582667282</v>
       </c>
       <c r="G12" t="n">
         <v>476670336</v>

</xml_diff>